<commit_message>
chore(import): regenerate Excel templates in the user's language
- generate_templates.py: OUT_DIR dò ngược thư mục gốc thay vì đếm cứng
  số '..' (script từng bị di chuyển và ghi template ra thư mục ma)
- banner + vùng dropdown cùng trỏ HÀNG 6; trước ghi 'từ hàng 5' nên người
  dùng ghi đè hàng ví dụ và dòng đầu bị nuốt im lặng
- mô tả cột Link nhắc 'điền TÊN, không điền mã'; dropdown cột Select in
  nhãn tiếng Việt thay enum tiếng Anh
- nhãn cột email người dùng: 'Email (Mã người dùng)' → 'Email đăng nhập'
- sinh lại 8 file .xlsx theo generator
</commit_message>
<xml_diff>
--- a/assetcore/public/import_templates/01a_danh_muc_tai_san.xlsx
+++ b/assetcore/public/import_templates/01a_danh_muc_tai_san.xlsx
@@ -547,7 +547,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>📋 HƯỚNG DẪN IMPORT: Danh mục tài sản (Category)  |  Điền dữ liệu từ hàng 5 trở xuống. Cột đỏ = bắt buộc. Không xóa hàng 2-4.</t>
+          <t>📋 HƯỚNG DẪN IMPORT: Danh mục tài sản (Category)  |  Điền dữ liệu từ HÀNG 6 trở xuống (hàng 5 là ví dụ mẫu, hệ thống bỏ qua). Cột đỏ = bắt buộc. Không xoá/không sửa hàng 1-5. Cột tham chiếu (danh mục, khoa phòng, vị trí, model, nhà cung cấp) điền TÊN, không điền mã.</t>
         </is>
       </c>
     </row>
@@ -720,7 +720,7 @@
       </c>
       <c r="I4" s="6" t="inlineStr">
         <is>
-          <t>Straight Line / Double Declining / Units of Production</t>
+          <t>Đường thẳng / Số dư giảm dần / Theo sản lượng.</t>
         </is>
       </c>
       <c r="J4" s="6" t="inlineStr">
@@ -782,7 +782,7 @@
       </c>
       <c r="I5" s="7" t="inlineStr">
         <is>
-          <t>Straight Line</t>
+          <t>Đường thẳng</t>
         </is>
       </c>
       <c r="J5" s="7" t="inlineStr">
@@ -2206,19 +2206,19 @@
     <mergeCell ref="A1:L1"/>
   </mergeCells>
   <dataValidations count="5">
-    <dataValidation sqref="E5:E105" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Giá trị không hợp lệ" error="Vui lòng chọn từ danh sách." type="list">
+    <dataValidation sqref="E6:E105" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Giá trị không hợp lệ" error="Vui lòng chọn từ danh sách." type="list">
       <formula1>"1,0"</formula1>
     </dataValidation>
-    <dataValidation sqref="G5:G105" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Giá trị không hợp lệ" error="Vui lòng chọn từ danh sách." type="list">
+    <dataValidation sqref="G6:G105" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Giá trị không hợp lệ" error="Vui lòng chọn từ danh sách." type="list">
       <formula1>"1,0"</formula1>
     </dataValidation>
-    <dataValidation sqref="I5:I105" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Giá trị không hợp lệ" error="Vui lòng chọn từ danh sách." type="list">
-      <formula1>"Straight Line,Double Declining,Units of Production"</formula1>
+    <dataValidation sqref="I6:I105" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Giá trị không hợp lệ" error="Vui lòng chọn từ danh sách." type="list">
+      <formula1>"Đường thẳng,Số dư giảm dần,Theo sản lượng"</formula1>
     </dataValidation>
-    <dataValidation sqref="K5:K105" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Giá trị không hợp lệ" error="Vui lòng chọn từ danh sách." type="list">
+    <dataValidation sqref="K6:K105" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Giá trị không hợp lệ" error="Vui lòng chọn từ danh sách." type="list">
       <formula1>"1,0"</formula1>
     </dataValidation>
-    <dataValidation sqref="L5:L105" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Giá trị không hợp lệ" error="Vui lòng chọn từ danh sách." type="list">
+    <dataValidation sqref="L6:L105" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Giá trị không hợp lệ" error="Vui lòng chọn từ danh sách." type="list">
       <formula1>"1,0"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>